<commit_message>
Allow rendering blocks inside other blocks of ruletext
</commit_message>
<xml_diff>
--- a/data/raw/rules/translations.xlsx
+++ b/data/raw/rules/translations.xlsx
@@ -2235,7 +2235,7 @@
   <si>
     <t xml:space="preserve">When a &lt;b&gt;Monster&lt;/b&gt; wishes to use this Brutal Power Attack, it must nominate a single enemy model involved in the Combat before models Back Away – this is the model that will be Hurled. A &lt;b&gt;Monster&lt;/b&gt; cannot nominate a model to be Hurled that has a Strength equal to or higher than their own. Then, all other enemy models (not the nominated model) Back Away as normal. The Monster will then Hurl the nominated model.
 To Hurl a model, follow the steps below:
-&lt;ul&gt;
+&lt;ol&gt;
 &lt;li&gt; The &lt;b&gt;Monster&lt;/b&gt; rolls a D3 and adds the difference in Strength between the &lt;b&gt;Monster&lt;/b&gt; and the nominated model – this is the Hurl Distance.&lt;/li&gt;
 &lt;li&gt;The &lt;b&gt;Monster&lt;/b&gt; must then take an Intelligence Test (if the &lt;b&gt;Monster&lt;/b&gt; is also a &lt;b&gt;Mount&lt;/b&gt;, it may use the Intelligence of its rider if it is better).&lt;/li&gt;
 &lt;li&gt;If the test is passed, the &lt;b&gt;Monster&lt;/b&gt; chooses an enemy model it can draw Line of Sight to, and within the Hurl Distance from itself, to Hurl the nominated model at – this is the target. A model can only be chosen as the target of a Hurl once per turn. If the test was failed, the opposing player may choose one of their models in Line of Sight of the &lt;b&gt;Monster&lt;/b&gt;, and within the Hurl Distance, to be the target instead.&lt;/li&gt;
@@ -2244,7 +2244,7 @@
 &lt;li&gt;The target model is then knocked Prone, if it has a Strength of 5 or less, and will suffer one Strength 6 hit (if it is a &lt;b&gt;Cavalry&lt;/b&gt; model then both rider and &lt;b&gt;Mount&lt;/b&gt; will suffer these hits). If it is a &lt;b&gt;Cavalry&lt;/b&gt; model then it is also Knocked Flying.&lt;/li&gt;
 &lt;li&gt;If there are no enemy models eligible to be the target, then the &lt;b&gt;Monster&lt;/b&gt; may choose a point on the battlefield it can draw Line of Sight within the Hurl Distance instead. Place the Hurled model on the chosen point; it is then knocked Prone and suffers two Strength 6 hits.&lt;/li&gt;
 &lt;li&gt;Once a &lt;b&gt;Monster&lt;/b&gt; model has used a Hurl, the Combat immediately ends and no further Strikes or Brutal Power Attacks can be made. A Monster cannot Hurl in the same turn in which it participates in a Heroic Combat.&lt;/li&gt;
-&lt;/ul&gt;</t>
+&lt;/ol&gt;</t>
   </si>
   <si>
     <t xml:space="preserve">hand-weapon.name</t>
@@ -2375,10 +2375,38 @@
     <t xml:space="preserve">elven-weapon.description</t>
   </si>
   <si>
-    <t xml:space="preserve">Some weapons will be described as an Elven weapon; for example, a model may have an Elven hand weapon or an Elven two-handed weapon.
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Some weapons will be described as an Elven weapon; for example, a model may have an Elven &lt;rule id="hand-weapon"&gt;hand weapon&lt;/rule&gt; or an Elven </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">&lt;rule id="two-handed-hand-weapon"&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">two-handed weapon&lt;/rule&gt;.
 If a model fights with an Elven weapon in a Combat, they will be more likely to win the Duel Roll in the result of a Drawn Combat. In these instances, a Good model armed with an Elven weapon will win the roll-off ona 3+, whilst an Evil model armed with an Elven weapon will win the roll-off on a 1-4. If both sides have an Elven weapon, neither side gains the benefit.
 Some Missile Weapons may also be classed as Elven weapons; however, the above bonus only applies to Melee Weapons as a model cannot choose to fight with a Missile Weapon in a Combat.
 Any weapon with the word ‘Elf’ in its name is automatically considered to be an Elven weapon.</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">master-forged.name</t>
@@ -2428,7 +2456,7 @@
   </si>
   <si>
     <t xml:space="preserve">A model with a throwing weapon can make a Shooting Attack with it in the Shoot Phase, even if it Moved its full Move Value in the preceding Move Phase.
-Alternatively, once per turn, a model may make a Shooting Attack with a throwing weapon during the Move Phaseas it Charges an enemy model. If a model wishes to use a throwing weapon in this manner, then when it Charges it will stop 1" away from the model it wishes to Charge, andthen make a Shooting Attack against the model. If the model using the throwing weapon begins its Move within the Control Zone of an enemy model it wishes to Charge, then it doesn’t need to Move first before throwing the weapon. This is made using all the normal rules for a Shooting Attack, with the exception of that throwing weapons thrown in this manner do not suffer the -1 penalty To Hit for Moving and Shooting.
+Alternatively, once per turn, a model may make a Shooting Attack with a throwing weapon during the Move Phase as it Charges an enemy model. If a model wishes to use a throwing weapon in this manner, then when it Charges it will stop 1" away from the model it wishes to Charge, and then make a Shooting Attack against the model. If the model using the throwing weapon begins its Move within the Control Zone of an enemy model it wishes to Charge, then it doesn’t need to Move first before throwing the weapon. This is made using all the normal rules for a Shooting Attack, with the exception of that throwing weapons thrown in this manner do not suffer the -1 penalty To Hit for Moving and Shooting.
 If the target is not slain, then the model continues their Charge as normal and must Charge the target of their Shooting Attack. If the target is slain, then the model may continue to Move as normal, and may even Charge a different target if they wish.
 Throwing weapons do not count towards an Army’s Bow Limit. However, an Army can only have one third of its models armed with throwing weapons, unless specifically stated otherwise.
 Throwing spears follow the same rules as throwing weapons, but have a slightly different profile, as shown on the Missile Weapon Chart.</t>
@@ -2498,7 +2526,7 @@
     <t xml:space="preserve">elven-cloak.description</t>
   </si>
   <si>
-    <t xml:space="preserve">A model wearing an Elven cloak has the Stalk Unseen special rule. Additionally, models targeting an &lt;b&gt;Infantry&lt;/b&gt; model wearing an Elven cloak with a Shooting Attack suffer a -1 penalty when rolling To Hit.</t>
+    <t xml:space="preserve">A model wearing an Elven cloak has the &lt;rule id="stalk-unseen"&gt;Stalk Unseen&lt;/rule&gt; special rule. Additionally, models targeting an &lt;b&gt;Infantry&lt;/b&gt; model wearing an Elven cloak with a Shooting Attack suffer a -1 penalty when rolling To Hit.</t>
   </si>
   <si>
     <t xml:space="preserve">war-drum.name</t>
@@ -4392,7 +4420,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="207" customFormat="false" ht="142.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="207" customFormat="false" ht="157.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A207" s="2" t="s">
         <v>412</v>
       </c>

</xml_diff>